<commit_message>
Working for discrete labeling
</commit_message>
<xml_diff>
--- a/data/baseline.xlsx
+++ b/data/baseline.xlsx
@@ -413,43 +413,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Column</t>
+          <t>col</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Sheet 1</t>
+          <t>sheet 1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Sheet 2</t>
+          <t>sheet 2</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>P-Value</t>
+          <t>pval</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>category</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>type</t>
         </is>
       </c>
     </row>
@@ -525,31 +525,15 @@
           <t>raceethnic</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>3 (15.79%)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>3 (10.34%)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>6 (12.50%)</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>0.28</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>black</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -560,23 +544,23 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1 (5.26%)</t>
+          <t>3 (15.79%)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6 (20.69%)</t>
+          <t>3 (10.34%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7 (14.58%)</t>
+          <t>6 (12.50%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>black</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -589,91 +573,75 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>15 (78.95%)</t>
+          <t>1 (5.26%)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20 (68.97%)</t>
+          <t>6 (20.69%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>35 (72.92%)</t>
+          <t>7 (14.58%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15 (78.95%)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>20 (68.97%)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>35 (72.92%)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>white</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>categorical</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>diabetes</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
         <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>categorical</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -681,31 +649,23 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>HTN</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>19 (100.00%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>28 (96.55%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0.39</t>
-        </is>
-      </c>
+          <t>47 (97.92%)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>0</t>
@@ -726,12 +686,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (3.45%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (2.08%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -747,28 +707,20 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>1 (5.26%)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1 (2.08%)</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>131/72 ?</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HTN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.39</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -776,31 +728,23 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>15 (78.95%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>24 (82.76%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
+          <t>39 (81.25%)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>0</t>
@@ -816,17 +760,17 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>3 (15.79%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>5 (17.24%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>8 (16.67%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -842,34 +786,26 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>tobacco_history</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
+          <t>1 (5.26%)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>0 (0.00%)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0.62</t>
-        </is>
-      </c>
+          <t>1 (2.08%)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>131/72 ?</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -879,28 +815,20 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -911,23 +839,23 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>5 (26.32%)</t>
+          <t>14 (73.68%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10 (34.48%)</t>
+          <t>29 (100.00%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15 (31.25%)</t>
+          <t>43 (89.58%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>former</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -937,34 +865,26 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>alcohol_history</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
+          <t>5 (26.32%)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>0 (0.00%)</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0.21</t>
-        </is>
-      </c>
+          <t>5 (10.42%)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -974,28 +894,20 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tobacco_history</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.62</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1006,23 +918,23 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>13 (68.42%)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1 (3.57%)</t>
+          <t>16 (55.17%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1 (2.13%)</t>
+          <t>29 (60.42%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1035,23 +947,23 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (5.26%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1 (3.57%)</t>
+          <t>3 (10.34%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1 (2.13%)</t>
+          <t>4 (8.33%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>socially</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1061,34 +973,26 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>pre-pec</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>5 (26.32%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>10 (34.48%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>0.67</t>
-        </is>
-      </c>
+          <t>15 (31.25%)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>former</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1098,28 +1002,20 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>alcohol_history</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>0.21</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1127,31 +1023,23 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>sub-pec</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>11 (57.89%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>9 (32.14%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0.67</t>
-        </is>
-      </c>
+          <t>20 (42.55%)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>0</t>
@@ -1167,17 +1055,17 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>8 (42.11%)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>17 (60.71%)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>25 (53.19%)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -1193,11 +1081,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>NSM</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>0 (0.00%)</t>
@@ -1205,22 +1089,18 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (3.57%)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+          <t>1 (2.13%)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1238,18 +1118,18 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (3.57%)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (2.13%)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>socially</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1261,34 +1141,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SSM</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
+          <t>pre-pec</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>0.67</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1299,62 +1163,54 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>4 (21.05%)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>9 (31.03%)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>13 (27.08%)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15 (78.95%)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>20 (68.97%)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>35 (72.92%)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>categorical</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>neoadjuvant chemotherapy (yes=1)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>0.99</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1362,28 +1218,20 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>sub-pec</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0.67</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1391,31 +1239,23 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>adjuvant chemotherapy (yes=1)</t>
-        </is>
-      </c>
+      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>15 (78.95%)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>20 (68.97%)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
-      </c>
+          <t>35 (72.92%)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>0</t>
@@ -1431,17 +1271,17 @@
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>4 (21.05%)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>9 (31.03%)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>13 (27.08%)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1459,34 +1299,18 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>immunotherapy (keytruda?)</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
+          <t>NSM</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1497,62 +1321,54 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>2 (10.53%)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>16 (55.17%)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>18 (37.50%)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17 (89.47%)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>13 (44.83%)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>30 (62.50%)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>categorical</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>RT (yes=1)</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>0.32</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1560,28 +1376,20 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SSM</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1589,31 +1397,23 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>adjuvant endocrine</t>
-        </is>
-      </c>
+      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>17 (89.47%)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>13 (44.83%)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
+          <t>30 (62.50%)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>0</t>
@@ -1629,17 +1429,17 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>2 (10.53%)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>16 (55.17%)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>18 (37.50%)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1657,34 +1457,18 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ADM/dermal sling</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
+          <t>neoadjuvant chemotherapy (yes=1)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1695,62 +1479,54 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>12 (63.16%)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>17 (58.62%)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>29 (60.42%)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>7 (36.84%)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>12 (41.38%)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>19 (39.58%)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>categorical</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>SLNB (yes=1)</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
       <c r="G41" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1758,28 +1534,20 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>adjuvant chemotherapy (yes=1)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>0.08</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1787,34 +1555,26 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ALND (yes=1)</t>
-        </is>
-      </c>
+      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>16 (84.21%)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>16 (55.17%)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>0.29</t>
-        </is>
-      </c>
+          <t>32 (66.67%)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1827,23 +1587,23 @@
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>3 (15.79%)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>13 (44.83%)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>16 (33.33%)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1855,34 +1615,18 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ER +</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
+          <t>immunotherapy (keytruda?)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>0.65</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1893,23 +1637,23 @@
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>17 (89.47%)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>25 (86.21%)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>42 (87.50%)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1919,34 +1663,26 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>PR+</t>
-        </is>
-      </c>
+      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>2 (10.53%)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>4 (13.79%)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>0.73</t>
-        </is>
-      </c>
+          <t>6 (12.50%)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -1956,28 +1692,20 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>RT (yes=1)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>0.32</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -1985,34 +1713,26 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>HER2+</t>
-        </is>
-      </c>
+      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>14 (73.68%)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>16 (55.17%)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
+          <t>30 (62.50%)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2025,23 +1745,23 @@
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>5 (26.32%)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>13 (44.83%)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>18 (37.50%)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2053,34 +1773,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>grade1</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>1 (7.69%)</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>1 (3.70%)</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2 (5.00%)</t>
-        </is>
-      </c>
+          <t>adjuvant endocrine</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0.52</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -2091,23 +1795,23 @@
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>8 (42.11%)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1 (3.70%)</t>
+          <t>12 (41.38%)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>1 (2.50%)</t>
+          <t>20 (41.67%)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">I </t>
+          <t>0</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2120,23 +1824,23 @@
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
-          <t>4 (30.77%)</t>
+          <t>11 (57.89%)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>13 (48.15%)</t>
+          <t>17 (58.62%)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>17 (42.50%)</t>
+          <t>28 (58.33%)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2146,28 +1850,20 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>6 (46.15%)</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>10 (37.04%)</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>16 (40.00%)</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>III</t>
-        </is>
-      </c>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ADM/dermal sling</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -2178,23 +1874,23 @@
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1 (7.69%)</t>
+          <t>0 (0.00%)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (3.45%)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>1 (2.50%)</t>
+          <t>1 (2.08%)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2207,23 +1903,23 @@
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1 (7.69%)</t>
+          <t>19 (100.00%)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1 (3.70%)</t>
+          <t>28 (96.55%)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2 (5.00%)</t>
+          <t>47 (97.92%)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2233,63 +1929,47 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SLNB (yes=1)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1 (6.25%)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
         <is>
           <t>0 (0.00%)</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>1 (3.70%)</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>1 (2.50%)</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>categorical</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>mastectomy laterality</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>0.96</t>
-        </is>
-      </c>
+          <t>3 (6.67%)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2302,23 +1982,23 @@
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
+          <t>15 (93.75%)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
           <t>0 (0.00%)</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>42 (93.33%)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2328,60 +2008,44 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ALND (yes=1)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>0.29</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>14 (87.50%)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
         <is>
           <t>0 (0.00%)</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>categorical</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>cancer laterality R(0), L (1), both (2)</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>0.37</t>
-        </is>
-      </c>
+          <t>35 (77.78%)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>0.0</t>
@@ -2397,17 +2061,17 @@
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
+          <t>2 (12.50%)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
           <t>0 (0.00%)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>10 (22.22%)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2423,28 +2087,20 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ER +</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -2452,34 +2108,26 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>clinical stage</t>
-        </is>
-      </c>
+      <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>3 (20.00%)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>3 (11.11%)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+          <t>6 (14.29%)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2492,23 +2140,23 @@
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>12 (80.00%)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>9 (34.62%)</t>
+          <t>24 (88.89%)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>9 (21.95%)</t>
+          <t>36 (85.71%)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2518,28 +2166,20 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>5 (33.33%)</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>5 (12.20%)</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IA </t>
-        </is>
-      </c>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>PR+</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -2555,18 +2195,18 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>5 (19.23%)</t>
+          <t>10 (37.04%)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>9 (21.95%)</t>
+          <t>14 (33.33%)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>IIA</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2579,23 +2219,23 @@
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
-          <t>1 (6.67%)</t>
+          <t>11 (73.33%)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>17 (62.96%)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>1 (2.44%)</t>
+          <t>28 (66.67%)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">IIA </t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2605,28 +2245,20 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1 (6.67%)</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>2 (7.69%)</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>3 (7.32%)</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>IIB</t>
-        </is>
-      </c>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>HER2+</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -2637,23 +2269,23 @@
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
-          <t>1 (6.67%)</t>
+          <t>12 (85.71%)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>3 (11.54%)</t>
+          <t>22 (81.48%)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>4 (9.76%)</t>
+          <t>34 (82.93%)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>IIIA</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2666,23 +2298,23 @@
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>2 (14.29%)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>1 (3.85%)</t>
+          <t>5 (18.52%)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>1 (2.44%)</t>
+          <t>7 (17.07%)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>T1N0M0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2694,34 +2326,18 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>cancer type</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>1 (5.26%)</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>5 (17.24%)</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>6 (12.50%)</t>
-        </is>
-      </c>
+          <t>grade1</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>0.30</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>DCIS</t>
-        </is>
-      </c>
+          <t>0.52</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -2732,23 +2348,23 @@
       <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
-          <t>1 (5.26%)</t>
+          <t>1 (7.69%)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>1 (3.45%)</t>
+          <t>1 (3.70%)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2 (4.17%)</t>
+          <t>2 (5.00%)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>DCIS, ADH</t>
+          <t>I</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2761,23 +2377,23 @@
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
-          <t>1 (5.26%)</t>
+          <t>0 (0.00%)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (3.70%)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>1 (2.08%)</t>
+          <t>1 (2.50%)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>DCIS, IDC</t>
+          <t xml:space="preserve">I </t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2790,23 +2406,23 @@
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
-          <t>1 (5.26%)</t>
+          <t>4 (30.77%)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>13 (48.15%)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>1 (2.08%)</t>
+          <t>17 (42.50%)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>DCIS, Paget's</t>
+          <t>II</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2819,23 +2435,23 @@
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
-          <t>7 (36.84%)</t>
+          <t>6 (46.15%)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16 (55.17%)</t>
+          <t>10 (37.04%)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>23 (47.92%)</t>
+          <t>16 (40.00%)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>IDC</t>
+          <t>III</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2848,23 +2464,23 @@
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
-          <t>1 (5.26%)</t>
+          <t>1 (7.69%)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2 (6.90%)</t>
+          <t>0 (0.00%)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>3 (6.25%)</t>
+          <t>1 (2.50%)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>IDC, DCIS</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2877,23 +2493,23 @@
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
-          <t>0 (0.00%)</t>
+          <t>1 (7.69%)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>1 (3.45%)</t>
+          <t>1 (3.70%)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>1 (2.08%)</t>
+          <t>2 (5.00%)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>IDC,DCIS</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2906,23 +2522,23 @@
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
-          <t>3 (15.79%)</t>
+          <t>0 (0.00%)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2 (6.90%)</t>
+          <t>1 (3.70%)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>5 (10.42%)</t>
+          <t>1 (2.50%)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>ILC</t>
+          <t>low</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2932,28 +2548,20 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>1 (5.26%)</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>0 (0.00%)</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>1 (2.08%)</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>LCIS</t>
-        </is>
-      </c>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>mastectomy laterality</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>categorical</t>
@@ -2964,26 +2572,756 @@
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
-          <t>3 (15.79%)</t>
+          <t>4 (21.05%)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2 (6.90%)</t>
+          <t>7 (24.14%)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>5 (10.42%)</t>
+          <t>11 (22.92%)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>3 (15.79%)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>4 (13.79%)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>7 (14.58%)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>12 (63.16%)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>18 (62.07%)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>30 (62.50%)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>cancer laterality R(0), L (1), both (2)</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>0.37</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10 (58.82%)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>16 (59.26%)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>26 (59.09%)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>6 (35.29%)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>11 (40.74%)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>17 (38.64%)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1 (5.88%)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>1 (2.27%)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>clinical stage</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>3 (20.00%)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>6 (23.08%)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>9 (21.95%)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr"/>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>9 (34.62%)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>9 (21.95%)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>5 (33.33%)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>5 (12.20%)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IA </t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>4 (26.67%)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>5 (19.23%)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>9 (21.95%)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>IIA</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1 (6.67%)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>1 (2.44%)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IIA </t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1 (6.67%)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2 (7.69%)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>3 (7.32%)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>IIB</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1 (6.67%)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>3 (11.54%)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>4 (9.76%)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>IIIA</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>1 (3.85%)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>1 (2.44%)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>T1N0M0</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>cancer type</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1 (5.26%)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>5 (17.24%)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>6 (12.50%)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>DCIS</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1 (5.26%)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>1 (3.45%)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>2 (4.17%)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>DCIS, ADH</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr"/>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1 (5.26%)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>1 (2.08%)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>DCIS, IDC</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr"/>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1 (5.26%)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>1 (2.08%)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>DCIS, Paget's</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr"/>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>7 (36.84%)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>16 (55.17%)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>23 (47.92%)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>IDC</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr"/>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1 (5.26%)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2 (6.90%)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>3 (6.25%)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>IDC, DCIS</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr"/>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>1 (3.45%)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>1 (2.08%)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>IDC,DCIS</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr"/>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>3 (15.79%)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2 (6.90%)</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>5 (10.42%)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>ILC</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr"/>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1 (5.26%)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>0 (0.00%)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>1 (2.08%)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>LCIS</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr"/>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>3 (15.79%)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2 (6.90%)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>5 (10.42%)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
           <t>prophylactic</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G107" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>

</xml_diff>